<commit_message>
Modifica post atribuicao de processos
</commit_message>
<xml_diff>
--- a/docs/robos/atribuicao_processo_sei/assets/Fila_de_Atribuicao.xlsx
+++ b/docs/robos/atribuicao_processo_sei/assets/Fila_de_Atribuicao.xlsx
@@ -1,24 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\m1528563\Downloads\testes\Arquivos_15_07_2025_14-41-32\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\x20151001\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1041F97-5941-4232-B135-5215D605A264}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74279D28-9CFC-4C4E-A4FB-ADC03DB12526}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2205" yWindow="2205" windowWidth="21600" windowHeight="11295" xr2:uid="{739A4E69-9282-4090-9AD2-5BE42687AA38}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{739A4E69-9282-4090-9AD2-5BE42687AA38}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -80,7 +91,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="8">
   <si>
     <t>CPF</t>
   </si>
@@ -92,6 +103,18 @@
   </si>
   <si>
     <t>Próxima Atribuição</t>
+  </si>
+  <si>
+    <t>a</t>
+  </si>
+  <si>
+    <t>b</t>
+  </si>
+  <si>
+    <t>c</t>
+  </si>
+  <si>
+    <t>123</t>
   </si>
 </sst>
 </file>
@@ -156,7 +179,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -240,35 +263,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -294,12 +293,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -309,24 +302,6 @@
   </cellStyles>
   <dxfs count="6">
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
@@ -350,6 +325,24 @@
         <left style="thin">
           <color auto="1"/>
         </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
         <right style="thin">
           <color auto="1"/>
         </right>
@@ -406,19 +399,15 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FFD52C3D-264E-4693-84B2-A8641405C546}" name="Tabela1" displayName="Tabela1" ref="A1:C41" totalsRowShown="0" headerRowBorderDxfId="5" tableBorderDxfId="4" totalsRowBorderDxfId="3">
-  <autoFilter ref="A1:C41" xr:uid="{FFD52C3D-264E-4693-84B2-A8641405C546}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FFD52C3D-264E-4693-84B2-A8641405C546}" name="Tabela1" displayName="Tabela1" ref="A1:C4" totalsRowShown="0" headerRowBorderDxfId="5" tableBorderDxfId="4" totalsRowBorderDxfId="3">
+  <autoFilter ref="A1:C4" xr:uid="{FFD52C3D-264E-4693-84B2-A8641405C546}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{A4C64A02-227D-4743-B9C0-8BE53D8FF732}" name="Número" dataDxfId="0">
+    <tableColumn id="1" xr3:uid="{A4C64A02-227D-4743-B9C0-8BE53D8FF732}" name="Número" dataDxfId="2">
       <calculatedColumnFormula>IF(B1&lt;&gt;"",SUM(A1+1),"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{D31C2692-8265-4B5E-8013-471FFD1678C8}" name="Nome" dataDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{DEFAFD7D-55FC-4785-A09F-4F7C6165A90E}" name="CPF" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{D31C2692-8265-4B5E-8013-471FFD1678C8}" name="Nome" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{DEFAFD7D-55FC-4785-A09F-4F7C6165A90E}" name="CPF" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -741,7 +730,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22A18A24-B3AF-479E-8112-79C6E2D54103}">
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.28515625" customWidth="1"/>
@@ -760,332 +749,48 @@
       <c r="C1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="9" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="str">
+      <c r="A2" s="4">
         <f>IF(B2&lt;&gt;"",SUM(1),"")</f>
-        <v/>
-      </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="5"/>
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>7</v>
+      </c>
       <c r="E2" s="2">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="str">
+      <c r="A3" s="4">
         <f>IF(B3&lt;&gt;"",A2+1,"")</f>
-        <v/>
-      </c>
-      <c r="B3" s="3"/>
-      <c r="C3" s="5"/>
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="4" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="str">
-        <f t="shared" ref="A4:A41" si="0">IF(B4&lt;&gt;"",A3+1,"")</f>
-        <v/>
-      </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="5"/>
-    </row>
-    <row r="5" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="B5" s="3"/>
-      <c r="C5" s="5"/>
-    </row>
-    <row r="6" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="B6" s="3"/>
-      <c r="C6" s="5"/>
-    </row>
-    <row r="7" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="B7" s="3"/>
-      <c r="C7" s="5"/>
-    </row>
-    <row r="8" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="B8" s="3"/>
-      <c r="C8" s="5"/>
-    </row>
-    <row r="9" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="B9" s="3"/>
-      <c r="C9" s="5"/>
-    </row>
-    <row r="10" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="B10" s="3"/>
-      <c r="C10" s="5"/>
-    </row>
-    <row r="11" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="B11" s="3"/>
-      <c r="C11" s="5"/>
-    </row>
-    <row r="12" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="B12" s="3"/>
-      <c r="C12" s="5"/>
-    </row>
-    <row r="13" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="B13" s="3"/>
-      <c r="C13" s="5"/>
-    </row>
-    <row r="14" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="B14" s="3"/>
-      <c r="C14" s="5"/>
-    </row>
-    <row r="15" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="B15" s="3"/>
-      <c r="C15" s="5"/>
-    </row>
-    <row r="16" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="B16" s="3"/>
-      <c r="C16" s="5"/>
-    </row>
-    <row r="17" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="B17" s="3"/>
-      <c r="C17" s="5"/>
-    </row>
-    <row r="18" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="B18" s="3"/>
-      <c r="C18" s="5"/>
-    </row>
-    <row r="19" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="B19" s="3"/>
-      <c r="C19" s="5"/>
-    </row>
-    <row r="20" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="B20" s="3"/>
-      <c r="C20" s="5"/>
-    </row>
-    <row r="21" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="B21" s="3"/>
-      <c r="C21" s="5"/>
-    </row>
-    <row r="22" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="B22" s="3"/>
-      <c r="C22" s="5"/>
-    </row>
-    <row r="23" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="B23" s="3"/>
-      <c r="C23" s="5"/>
-    </row>
-    <row r="24" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="B24" s="3"/>
-      <c r="C24" s="5"/>
-    </row>
-    <row r="25" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="B25" s="3"/>
-      <c r="C25" s="5"/>
-    </row>
-    <row r="26" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="B26" s="3"/>
-      <c r="C26" s="5"/>
-    </row>
-    <row r="27" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="B27" s="3"/>
-      <c r="C27" s="5"/>
-    </row>
-    <row r="28" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="B28" s="3"/>
-      <c r="C28" s="5"/>
-    </row>
-    <row r="29" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="B29" s="9"/>
-      <c r="C29" s="10"/>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="B30" s="3"/>
-      <c r="C30" s="5"/>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="B31" s="3"/>
-      <c r="C31" s="5"/>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="B32" s="3"/>
-      <c r="C32" s="5"/>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="B33" s="3"/>
-      <c r="C33" s="5"/>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A34" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="B34" s="3"/>
-      <c r="C34" s="5"/>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="B35" s="3"/>
-      <c r="C35" s="5"/>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="B36" s="3"/>
-      <c r="C36" s="5"/>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="B37" s="3"/>
-      <c r="C37" s="5"/>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A38" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="B38" s="3"/>
-      <c r="C38" s="5"/>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="B39" s="3"/>
-      <c r="C39" s="5"/>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A40" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="B40" s="3"/>
-      <c r="C40" s="5"/>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A41" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="B41" s="9"/>
-      <c r="C41" s="10"/>
+      <c r="A4" s="4">
+        <f t="shared" ref="A4" si="0">IF(B4&lt;&gt;"",A3+1,"")</f>
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>7</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>